<commit_message>
Update lectures 8–15 and revise course schedule
- Revise lecture content, announcements, and R demos
- Add Lecture 15 Demo 2
- Update quiz dates, calendars, weekly schedules, and syllabus
</commit_message>
<xml_diff>
--- a/materials/generated_outputs/Weekly Schedules.xlsx
+++ b/materials/generated_outputs/Weekly Schedules.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="AutoGenerated Schedule" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AutoGenerated Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -653,12 +653,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Quiz 2, Lecture 16, Lecture 17</t>
+          <t>Lecture 16, Lecture 17, Lecture 18</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Quiz 2: in the lecture time; Lecture 16: Point estimates and sampling variability, continued (Chapter 5.1); Lecture 17: Confidence intervals (Chapter 5.2)</t>
+          <t>Lecture 16: Point estimates and sampling variability, continued (Chapter 5.1); Lecture 17: Confidence intervals (Chapter 5.2); Lecture 18: Hypothesis testing for a proportion (Chapter 5.3)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -670,7 +670,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Quiz 2: Near Indigenous People's Day Holiday, Classes Suspended | Quiz 2: Substitute a Monday schedule of classes | Lecture 16: Near Indigenous People's Day Holiday, Classes Suspended | Lecture 16: Near Substitute a Monday schedule of classes</t>
+          <t>Lecture 16: Near Indigenous People's Day Holiday, Classes Suspended | Lecture 16: Substitute a Monday schedule of classes | Lecture 17: Near Indigenous People's Day Holiday, Classes Suspended | Lecture 17: Near Substitute a Monday schedule of classes</t>
         </is>
       </c>
     </row>
@@ -680,12 +680,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lecture 18, Lecture 19, Lecture 20</t>
+          <t>Quiz 2, Lecture 19, Lecture 20</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Lecture 18: Hypothesis testing for a proportion (Chapter 5.3); Lecture 19: Hypothesis testing for a proportion, continued (Chapter 5.3); Lecture 20: Inference for a single proportion (Chapter 6.1)</t>
+          <t>Quiz 2: in the lecture time; Lecture 19: Hypothesis testing for a proportion, continued (Chapter 5.3); Lecture 20: Inference for a single proportion (Chapter 6.1)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Quiz 3: tentative; Lecture 24: One-sample means with the t-distribution (Chapter 7.1); Lecture 25: CIs for one-sample means, Paired data (Chapter 7.2)</t>
+          <t>Quiz 3: in the lecture time; Lecture 24: One-sample means with the t-distribution (Chapter 7.1); Lecture 25: CIs for one-sample means, Paired data (Chapter 7.2)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Quiz 4: tentative</t>
+          <t>Quiz 4: in the lecture time</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Lecture 35: Case study in modern statistical modeling; Quiz 5: tentative; Lecture 36: Wrap-up and evaluations</t>
+          <t>Lecture 35: Case study in modern statistical modeling; Quiz 5: in the lecture time; Lecture 36: Wrap-up and evaluations</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>

</xml_diff>